<commit_message>
edycja kodów i dodanie pliku z wykresami
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\studia_aisd\algorytmy_sortowania\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3432E9FB-6B9B-41D5-8434-8BEA55D4FAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9053E167-0B17-454B-A621-07782CA8E03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B75CB99-AA71-4B89-8348-2D877F97A134}"/>
   </bookViews>
@@ -39,8 +39,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="#,##0.000_ ;\-#,##0.000\ "/>
-    <numFmt numFmtId="170" formatCode="#,##0.00000_ ;\-#,##0.00000\ "/>
+    <numFmt numFmtId="164" formatCode="#,##0.000_ ;\-#,##0.000\ "/>
+    <numFmt numFmtId="165" formatCode="#,##0.00000_ ;\-#,##0.00000\ "/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -91,9 +91,9 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -195,9 +195,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="16"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
                 </c:pt>
@@ -252,53 +249,50 @@
               <c:numCache>
                 <c:formatCode>#\ ##0.00000_ ;\-#\ ##0.00000\ </c:formatCode>
                 <c:ptCount val="16"/>
-                <c:pt idx="0" formatCode="General">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.2903599999845E-2</c:v>
+                  <c:v>1.2895630000002699E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.1334100000531097E-2</c:v>
+                  <c:v>4.5536090000041399E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.111546400000406</c:v>
+                  <c:v>0.10659839999998399</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.22205050000047699</c:v>
+                  <c:v>0.17843498000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.325638600000274</c:v>
+                  <c:v>0.27907319000005298</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.46151140000074498</c:v>
+                  <c:v>0.39907955999997202</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.61490050000065799</c:v>
+                  <c:v>0.54504456000004198</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.77242959999966798</c:v>
+                  <c:v>0.71580754000005897</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.965670399999908</c:v>
+                  <c:v>0.908800730000075</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.1699397000002101</c:v>
+                  <c:v>1.1198589000000501</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.4155937000004899</c:v>
+                  <c:v>1.35082415000006</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.69318070000008</c:v>
+                  <c:v>1.61096243000001</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.0177727999998698</c:v>
+                  <c:v>1.89438412999998</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2.3262781999992499</c:v>
+                  <c:v>2.2099056500000098</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2.6460499999999998</c:v>
+                  <c:v>2.5968066699999302</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -324,6 +318,7 @@
       <c:valAx>
         <c:axId val="723363720"/>
         <c:scaling>
+          <c:logBase val="2"/>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -512,6 +507,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pl-PL"/>
+              <a:t>IS</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -702,7 +722,9 @@
       <c:valAx>
         <c:axId val="763103208"/>
         <c:scaling>
+          <c:logBase val="2"/>
           <c:orientation val="minMax"/>
+          <c:min val="1"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -720,7 +742,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0\K" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -782,7 +804,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="#\ ##0.00000_ ;\-#\ ##0.00000\ " sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -822,6 +844,7 @@
         <c:crossAx val="763103208"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
+        <c:majorUnit val="0.2"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -2369,12 +2392,6 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
       <c r="G2" s="1"/>
       <c r="N2" t="s">
         <v>1</v>
@@ -2385,10 +2402,14 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <v>1.2903599999845E-2</v>
+        <v>1.2895630000002699E-2</v>
       </c>
       <c r="B3">
         <v>1</v>
+      </c>
+      <c r="C3">
+        <f>B3*1000</f>
+        <v>1000</v>
       </c>
       <c r="N3" s="3">
         <v>1.29E-2</v>
@@ -2399,10 +2420,14 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>5.1334100000531097E-2</v>
+        <v>4.5536090000041399E-2</v>
       </c>
       <c r="B4">
         <v>2</v>
+      </c>
+      <c r="C4">
+        <f>B4*1000</f>
+        <v>2000</v>
       </c>
       <c r="N4" s="3">
         <v>5.1330000000000001E-2</v>
@@ -2413,10 +2438,14 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
-        <v>0.111546400000406</v>
+        <v>0.10659839999998399</v>
       </c>
       <c r="B5">
         <v>3</v>
+      </c>
+      <c r="C5">
+        <f t="shared" ref="C5:C17" si="0">B5*1000</f>
+        <v>3000</v>
       </c>
       <c r="N5" s="3">
         <v>0.11155</v>
@@ -2427,10 +2456,14 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
-        <v>0.22205050000047699</v>
+        <v>0.17843498000002</v>
       </c>
       <c r="B6">
         <v>4</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>4000</v>
       </c>
       <c r="N6" s="3">
         <v>0.22205</v>
@@ -2441,10 +2474,14 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <v>0.325638600000274</v>
+        <v>0.27907319000005298</v>
       </c>
       <c r="B7">
         <v>5</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>5000</v>
       </c>
       <c r="N7" s="3">
         <v>0.32563999999999999</v>
@@ -2455,10 +2492,14 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
-        <v>0.46151140000074498</v>
+        <v>0.39907955999997202</v>
       </c>
       <c r="B8">
         <v>6</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>6000</v>
       </c>
       <c r="N8" s="3">
         <v>0.46150999999999998</v>
@@ -2469,10 +2510,14 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
-        <v>0.61490050000065799</v>
+        <v>0.54504456000004198</v>
       </c>
       <c r="B9">
         <v>7</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>7000</v>
       </c>
       <c r="N9" s="3">
         <v>0.6149</v>
@@ -2483,10 +2528,14 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
-        <v>0.77242959999966798</v>
+        <v>0.71580754000005897</v>
       </c>
       <c r="B10">
         <v>8</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>8000</v>
       </c>
       <c r="N10" s="3">
         <v>0.77242999999999995</v>
@@ -2497,10 +2546,14 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
-        <v>0.965670399999908</v>
+        <v>0.908800730000075</v>
       </c>
       <c r="B11">
         <v>9</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>9000</v>
       </c>
       <c r="N11" s="3">
         <v>0.96567000000000003</v>
@@ -2511,10 +2564,14 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
-        <v>1.1699397000002101</v>
+        <v>1.1198589000000501</v>
       </c>
       <c r="B12">
         <v>10</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>10000</v>
       </c>
       <c r="N12" s="3">
         <v>1.16994</v>
@@ -2525,10 +2582,14 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
-        <v>1.4155937000004899</v>
+        <v>1.35082415000006</v>
       </c>
       <c r="B13">
         <v>11</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>11000</v>
       </c>
       <c r="N13" s="3">
         <v>1.4155899999999999</v>
@@ -2539,10 +2600,14 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
-        <v>1.69318070000008</v>
+        <v>1.61096243000001</v>
       </c>
       <c r="B14">
         <v>12</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>12000</v>
       </c>
       <c r="N14" s="3">
         <v>1.6931799999999999</v>
@@ -2553,10 +2618,14 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
-        <v>2.0177727999998698</v>
+        <v>1.89438412999998</v>
       </c>
       <c r="B15">
         <v>13</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>13000</v>
       </c>
       <c r="N15" s="3">
         <v>2.0177700000000001</v>
@@ -2567,10 +2636,14 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
-        <v>2.3262781999992499</v>
+        <v>2.2099056500000098</v>
       </c>
       <c r="B16">
         <v>14</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>14000</v>
       </c>
       <c r="N16" s="3">
         <v>2.3262800000000001</v>
@@ -2581,10 +2654,14 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
-        <v>2.6460499999999998</v>
+        <v>2.5968066699999302</v>
       </c>
       <c r="B17" s="4">
         <v>15</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>15000</v>
       </c>
       <c r="N17" s="2">
         <v>2.6460513000001802</v>

</xml_diff>